<commit_message>
save 25 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_13_JavaScript_sugarJS.xlsx
+++ b/4 четверть_13_JavaScript_sugarJS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F0778A-5208-4EE8-95EE-CF2997BF0BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F35D37-D427-4191-9ED9-5E9D52B741D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12315" yWindow="-18960" windowWidth="28770" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sugarjs" sheetId="20" r:id="rId1"/>
@@ -21067,7 +21067,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>46</v>
       </c>
@@ -24434,7 +24434,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="112" spans="1:23" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>205</v>
       </c>
@@ -24996,7 +24996,7 @@
       </c>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="1:23" s="2" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" s="2" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>341</v>
       </c>
@@ -25722,7 +25722,7 @@
       <c r="AA51" s="1"/>
       <c r="AB51" s="1"/>
     </row>
-    <row r="52" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>40</v>
       </c>
@@ -25757,7 +25757,7 @@
       <c r="V52" s="2"/>
       <c r="W52" s="1"/>
     </row>
-    <row r="53" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>121</v>
       </c>
@@ -25950,7 +25950,7 @@
       <c r="V58" s="2"/>
       <c r="W58" s="1"/>
     </row>
-    <row r="59" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A59" s="17" t="s">
         <v>332</v>
       </c>

</xml_diff>

<commit_message>
save 28 04 2026
</commit_message>
<xml_diff>
--- a/4 четверть_13_JavaScript_sugarJS.xlsx
+++ b/4 четверть_13_JavaScript_sugarJS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686A9354-FAAC-43A9-9B90-5BCFEC381F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE26399-7131-44D8-932C-91C05AA6019B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21205,7 +21205,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>45</v>
       </c>
@@ -24691,7 +24691,7 @@
       </c>
       <c r="B111" s="11"/>
     </row>
-    <row r="112" spans="1:24" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:24" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>202</v>
       </c>
@@ -25265,7 +25265,7 @@
       </c>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="1:23" s="2" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" s="2" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>338</v>
       </c>
@@ -25991,7 +25991,7 @@
       <c r="AA51" s="1"/>
       <c r="AB51" s="1"/>
     </row>
-    <row r="52" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>39</v>
       </c>
@@ -26026,7 +26026,7 @@
       <c r="V52" s="2"/>
       <c r="W52" s="1"/>
     </row>
-    <row r="53" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>120</v>
       </c>
@@ -26219,7 +26219,7 @@
       <c r="V58" s="2"/>
       <c r="W58" s="1"/>
     </row>
-    <row r="59" spans="1:28" s="4" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:28" s="4" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A59" s="17" t="s">
         <v>329</v>
       </c>

</xml_diff>

<commit_message>
save 20 05 2026
</commit_message>
<xml_diff>
--- a/4 четверть_13_JavaScript_sugarJS.xlsx
+++ b/4 четверть_13_JavaScript_sugarJS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB174D05-A0C6-4EB0-BB96-CF438A32CBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EACC82-AF8E-4C0E-93FF-DE353A550C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13875" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sugarjs" sheetId="20" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1356" uniqueCount="1094">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1356" uniqueCount="1096">
   <si>
     <t>construct(n,indexMapFn)</t>
   </si>
@@ -18607,17 +18607,133 @@
 users.least(true, 'profile.type') [&lt;User:Harry&gt;, &lt;User:Georgia&gt;]</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slice
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Аналог </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>to</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>если с аргументом</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slice
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Аналог </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>first</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>если с аргументом</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="35" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -18949,9 +19065,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -18962,50 +19078,50 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="19" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -19014,42 +19130,42 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -19064,6 +19180,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -20705,14 +20824,14 @@
     <row r="18" spans="1:23" s="20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="21"/>
       <c r="C18" s="21"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
       <c r="H18" s="21"/>
       <c r="Q18" s="21"/>
       <c r="R18" s="21"/>
       <c r="S18" s="21"/>
       <c r="T18" s="21"/>
-      <c r="U18" s="31"/>
+      <c r="U18" s="30"/>
       <c r="V18" s="21"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
@@ -20740,7 +20859,7 @@
       <c r="B20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="36" t="s">
+      <c r="C20" s="35" t="s">
         <v>903</v>
       </c>
       <c r="D20" s="2" t="s">
@@ -20774,7 +20893,7 @@
       <c r="B22" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="31" t="s">
         <v>1013</v>
       </c>
       <c r="D22" s="2" t="s">
@@ -20811,10 +20930,10 @@
       <c r="C24" s="25" t="s">
         <v>1016</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="31" t="s">
         <v>1015</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="E24" s="31" t="s">
         <v>963</v>
       </c>
     </row>
@@ -20828,10 +20947,10 @@
       <c r="C25" s="25" t="s">
         <v>1062</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="31" t="s">
         <v>1061</v>
       </c>
-      <c r="E25" s="32" t="s">
+      <c r="E25" s="31" t="s">
         <v>963</v>
       </c>
     </row>
@@ -20845,10 +20964,10 @@
       <c r="C26" s="2" t="s">
         <v>1063</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="31" t="s">
         <v>962</v>
       </c>
-      <c r="E26" s="32" t="s">
+      <c r="E26" s="31" t="s">
         <v>963</v>
       </c>
     </row>
@@ -20914,10 +21033,10 @@
       <c r="C31" s="25" t="s">
         <v>1065</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="D31" s="31" t="s">
         <v>1061</v>
       </c>
-      <c r="E31" s="32" t="s">
+      <c r="E31" s="31" t="s">
         <v>963</v>
       </c>
     </row>
@@ -21305,7 +21424,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>45</v>
       </c>
@@ -21343,7 +21462,7 @@
       <c r="B64" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C64" s="39" t="s">
+      <c r="C64" s="38" t="s">
         <v>1092</v>
       </c>
       <c r="D64" s="14" t="s">
@@ -21363,7 +21482,7 @@
       <c r="B66" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C66" s="38" t="s">
+      <c r="C66" s="37" t="s">
         <v>134</v>
       </c>
       <c r="D66" s="14" t="s">
@@ -21402,7 +21521,7 @@
       <c r="B69" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C69" s="38" t="s">
+      <c r="C69" s="37" t="s">
         <v>160</v>
       </c>
       <c r="D69" s="14" t="s">
@@ -21491,7 +21610,7 @@
       <c r="B76" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C76" s="37" t="s">
+      <c r="C76" s="36" t="s">
         <v>1080</v>
       </c>
       <c r="D76" s="14" t="s">
@@ -21742,7 +21861,7 @@
       <c r="B95" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C95" s="24" t="s">
+      <c r="C95" s="39" t="s">
         <v>137</v>
       </c>
       <c r="D95" s="14" t="s">
@@ -25002,10 +25121,10 @@
       <c r="D119" s="2" t="s">
         <v>938</v>
       </c>
-      <c r="E119" s="32" t="s">
+      <c r="E119" s="31" t="s">
         <v>937</v>
       </c>
-      <c r="F119" s="32" t="s">
+      <c r="F119" s="31" t="s">
         <v>939</v>
       </c>
     </row>
@@ -25017,10 +25136,10 @@
       <c r="D120" s="25" t="s">
         <v>942</v>
       </c>
-      <c r="E120" s="32" t="s">
+      <c r="E120" s="31" t="s">
         <v>941</v>
       </c>
-      <c r="F120" s="32" t="s">
+      <c r="F120" s="31" t="s">
         <v>943</v>
       </c>
     </row>
@@ -25032,7 +25151,7 @@
       <c r="D121" s="2" t="s">
         <v>948</v>
       </c>
-      <c r="E121" s="32" t="s">
+      <c r="E121" s="31" t="s">
         <v>945</v>
       </c>
     </row>
@@ -25041,13 +25160,13 @@
         <v>949</v>
       </c>
       <c r="B122" s="2"/>
-      <c r="D122" s="33" t="s">
+      <c r="D122" s="32" t="s">
         <v>951</v>
       </c>
-      <c r="E122" s="32" t="s">
+      <c r="E122" s="31" t="s">
         <v>950</v>
       </c>
-      <c r="F122" s="32" t="s">
+      <c r="F122" s="31" t="s">
         <v>952</v>
       </c>
     </row>
@@ -25059,10 +25178,10 @@
       <c r="D123" s="25" t="s">
         <v>955</v>
       </c>
-      <c r="E123" s="32" t="s">
+      <c r="E123" s="31" t="s">
         <v>954</v>
       </c>
-      <c r="F123" s="32" t="s">
+      <c r="F123" s="31" t="s">
         <v>956</v>
       </c>
     </row>
@@ -25121,7 +25240,7 @@
       <c r="F151" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -26060,7 +26179,7 @@
       <c r="A51" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="B51" s="36" t="s">
+      <c r="B51" s="35" t="s">
         <v>1073</v>
       </c>
       <c r="C51" s="2" t="s">
@@ -26095,7 +26214,7 @@
       <c r="A52" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B52" s="36" t="s">
+      <c r="B52" s="35" t="s">
         <v>1074</v>
       </c>
       <c r="C52" s="2" t="s">
@@ -26104,7 +26223,7 @@
       <c r="D52" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="E52" s="35" t="s">
+      <c r="E52" s="34" t="s">
         <v>329</v>
       </c>
       <c r="F52" s="7"/>
@@ -26130,7 +26249,7 @@
       <c r="A53" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B53" s="36" t="s">
+      <c r="B53" s="35" t="s">
         <v>1075</v>
       </c>
       <c r="C53" s="2" t="s">
@@ -27343,9 +27462,9 @@
         <v>725</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C31" s="29" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C31" s="40" t="s">
         <v>882</v>
       </c>
       <c r="D31" s="24" t="s">
@@ -27357,7 +27476,7 @@
         <v>806</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>143</v>
+        <v>1095</v>
       </c>
       <c r="C32" s="25" t="s">
         <v>883</v>
@@ -28183,7 +28302,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="33" t="s">
         <v>1021</v>
       </c>
     </row>
@@ -28286,7 +28405,7 @@
       <c r="B22" s="2" t="s">
         <v>1027</v>
       </c>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="36" t="s">
         <v>907</v>
       </c>
       <c r="D22" s="2" t="s">
@@ -28303,7 +28422,7 @@
       <c r="C23" s="2" t="s">
         <v>980</v>
       </c>
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="31" t="s">
         <v>979</v>
       </c>
     </row>
@@ -28317,7 +28436,7 @@
       <c r="C24" s="25" t="s">
         <v>983</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="31" t="s">
         <v>982</v>
       </c>
     </row>
@@ -28331,7 +28450,7 @@
       <c r="C25" s="2" t="s">
         <v>989</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="31" t="s">
         <v>988</v>
       </c>
     </row>
@@ -28345,7 +28464,7 @@
       <c r="C26" s="25" t="s">
         <v>986</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D26" s="31" t="s">
         <v>985</v>
       </c>
     </row>
@@ -28364,7 +28483,7 @@
       <c r="C28" s="2" t="s">
         <v>992</v>
       </c>
-      <c r="D28" s="32" t="s">
+      <c r="D28" s="31" t="s">
         <v>991</v>
       </c>
       <c r="E28" s="24"/>
@@ -28379,10 +28498,10 @@
       <c r="C29" s="25" t="s">
         <v>996</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="31" t="s">
         <v>993</v>
       </c>
-      <c r="E29" s="32" t="s">
+      <c r="E29" s="31" t="s">
         <v>995</v>
       </c>
     </row>
@@ -28398,7 +28517,7 @@
       <c r="A31" s="2" t="s">
         <v>911</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="31" t="s">
         <v>913</v>
       </c>
       <c r="D31" s="2" t="s">
@@ -28406,7 +28525,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A32" s="34" t="s">
+      <c r="A32" s="33" t="s">
         <v>1021</v>
       </c>
       <c r="B32" s="1"/>
@@ -28420,7 +28539,7 @@
       <c r="C33" s="25" t="s">
         <v>921</v>
       </c>
-      <c r="D33" s="32" t="s">
+      <c r="D33" s="31" t="s">
         <v>920</v>
       </c>
     </row>
@@ -28429,7 +28548,7 @@
         <v>1023</v>
       </c>
       <c r="C34" s="25"/>
-      <c r="D34" s="32"/>
+      <c r="D34" s="31"/>
     </row>
     <row r="35" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -28441,7 +28560,7 @@
       <c r="C35" s="25" t="s">
         <v>926</v>
       </c>
-      <c r="D35" s="32" t="s">
+      <c r="D35" s="31" t="s">
         <v>925</v>
       </c>
     </row>
@@ -28455,7 +28574,7 @@
       <c r="C36" s="25" t="s">
         <v>935</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="31" t="s">
         <v>934</v>
       </c>
     </row>
@@ -28464,7 +28583,7 @@
         <v>1022</v>
       </c>
       <c r="C37" s="25"/>
-      <c r="D37" s="32"/>
+      <c r="D37" s="31"/>
     </row>
     <row r="38" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
@@ -28476,7 +28595,7 @@
       <c r="C38" s="25" t="s">
         <v>971</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="31" t="s">
         <v>929</v>
       </c>
     </row>
@@ -28490,7 +28609,7 @@
       <c r="C39" s="2" t="s">
         <v>970</v>
       </c>
-      <c r="D39" s="32" t="s">
+      <c r="D39" s="31" t="s">
         <v>969</v>
       </c>
     </row>
@@ -28504,7 +28623,7 @@
       <c r="C40" s="25" t="s">
         <v>1008</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="D40" s="31" t="s">
         <v>1007</v>
       </c>
     </row>
@@ -28512,7 +28631,7 @@
       <c r="A41" s="15" t="s">
         <v>1025</v>
       </c>
-      <c r="D41" s="32"/>
+      <c r="D41" s="31"/>
     </row>
     <row r="42" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
@@ -28524,7 +28643,7 @@
       <c r="C42" s="25" t="s">
         <v>932</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D42" s="31" t="s">
         <v>931</v>
       </c>
     </row>
@@ -28533,7 +28652,7 @@
         <v>1038</v>
       </c>
       <c r="C43" s="25"/>
-      <c r="D43" s="32"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
@@ -28545,7 +28664,7 @@
       <c r="C44" s="2" t="s">
         <v>977</v>
       </c>
-      <c r="D44" s="32" t="s">
+      <c r="D44" s="31" t="s">
         <v>976</v>
       </c>
     </row>
@@ -28554,8 +28673,8 @@
         <v>1037</v>
       </c>
       <c r="C45" s="25"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
@@ -28567,7 +28686,7 @@
       <c r="C46" s="2" t="s">
         <v>999</v>
       </c>
-      <c r="D46" s="32" t="s">
+      <c r="D46" s="31" t="s">
         <v>998</v>
       </c>
     </row>
@@ -28581,7 +28700,7 @@
       <c r="C47" s="2" t="s">
         <v>974</v>
       </c>
-      <c r="D47" s="32" t="s">
+      <c r="D47" s="31" t="s">
         <v>973</v>
       </c>
     </row>
@@ -28595,7 +28714,7 @@
       <c r="C48" s="2" t="s">
         <v>967</v>
       </c>
-      <c r="D48" s="32" t="s">
+      <c r="D48" s="31" t="s">
         <v>966</v>
       </c>
     </row>
@@ -28609,7 +28728,7 @@
       <c r="C49" s="25" t="s">
         <v>1002</v>
       </c>
-      <c r="D49" s="32" t="s">
+      <c r="D49" s="31" t="s">
         <v>1001</v>
       </c>
       <c r="E49" s="1"/>
@@ -28624,7 +28743,7 @@
       <c r="C50" s="25" t="s">
         <v>1005</v>
       </c>
-      <c r="D50" s="32" t="s">
+      <c r="D50" s="31" t="s">
         <v>1004</v>
       </c>
       <c r="E50" s="1"/>
@@ -28639,7 +28758,7 @@
       <c r="C51" s="25" t="s">
         <v>924</v>
       </c>
-      <c r="D51" s="32" t="s">
+      <c r="D51" s="31" t="s">
         <v>923</v>
       </c>
     </row>
@@ -28661,7 +28780,7 @@
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="25"/>
-      <c r="D53" s="32"/>
+      <c r="D53" s="31"/>
       <c r="E53" s="4"/>
       <c r="G53" s="1"/>
       <c r="H53" s="2"/>
@@ -28683,7 +28802,7 @@
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="25"/>
-      <c r="D55" s="32"/>
+      <c r="D55" s="31"/>
       <c r="E55" s="4"/>
       <c r="G55" s="1"/>
       <c r="H55" s="2"/>
@@ -28704,7 +28823,7 @@
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="25"/>
-      <c r="D56" s="32"/>
+      <c r="D56" s="31"/>
       <c r="E56" s="4"/>
       <c r="G56" s="1"/>
       <c r="H56" s="2"/>
@@ -28725,7 +28844,7 @@
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="25"/>
-      <c r="D57" s="32"/>
+      <c r="D57" s="31"/>
       <c r="E57" s="4"/>
       <c r="G57" s="1"/>
       <c r="H57" s="2"/>
@@ -28746,7 +28865,7 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="25"/>
-      <c r="D58" s="32"/>
+      <c r="D58" s="31"/>
       <c r="E58" s="4"/>
       <c r="G58" s="1"/>
       <c r="H58" s="2"/>
@@ -28767,7 +28886,7 @@
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="25"/>
-      <c r="D59" s="32"/>
+      <c r="D59" s="31"/>
       <c r="E59" s="4"/>
       <c r="G59" s="1"/>
       <c r="H59" s="2"/>
@@ -28788,7 +28907,7 @@
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="25"/>
-      <c r="D60" s="32"/>
+      <c r="D60" s="31"/>
       <c r="E60" s="4"/>
       <c r="G60" s="1"/>
       <c r="H60" s="2"/>
@@ -28809,7 +28928,7 @@
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="25"/>
-      <c r="D61" s="32"/>
+      <c r="D61" s="31"/>
       <c r="E61" s="4"/>
       <c r="G61" s="1"/>
       <c r="H61" s="2"/>
@@ -28830,7 +28949,7 @@
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="25"/>
-      <c r="D62" s="32"/>
+      <c r="D62" s="31"/>
       <c r="E62" s="4"/>
       <c r="G62" s="1"/>
       <c r="H62" s="2"/>
@@ -28851,7 +28970,7 @@
       <c r="A63" s="2"/>
       <c r="B63" s="27"/>
       <c r="C63" s="25"/>
-      <c r="D63" s="32"/>
+      <c r="D63" s="31"/>
       <c r="E63" s="4"/>
       <c r="G63" s="1"/>
       <c r="H63" s="2"/>
@@ -28872,7 +28991,7 @@
       <c r="A64" s="2"/>
       <c r="B64" s="27"/>
       <c r="C64" s="25"/>
-      <c r="D64" s="32"/>
+      <c r="D64" s="31"/>
       <c r="E64" s="4"/>
       <c r="G64" s="1"/>
       <c r="H64" s="2"/>
@@ -28893,7 +29012,7 @@
       <c r="A65" s="2"/>
       <c r="B65" s="27"/>
       <c r="C65" s="25"/>
-      <c r="D65" s="32"/>
+      <c r="D65" s="31"/>
       <c r="E65" s="4"/>
       <c r="G65" s="1"/>
       <c r="H65" s="2"/>
@@ -28914,7 +29033,7 @@
       <c r="A66" s="2"/>
       <c r="B66" s="27"/>
       <c r="C66" s="26"/>
-      <c r="D66" s="32"/>
+      <c r="D66" s="31"/>
       <c r="E66" s="4"/>
       <c r="G66" s="1"/>
       <c r="H66" s="2"/>
@@ -28935,7 +29054,7 @@
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
-      <c r="D67" s="32"/>
+      <c r="D67" s="31"/>
       <c r="E67" s="4"/>
       <c r="G67" s="1"/>
       <c r="H67" s="2"/>
@@ -28956,7 +29075,7 @@
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="32"/>
+      <c r="D68" s="31"/>
       <c r="E68" s="4"/>
       <c r="G68" s="1"/>
       <c r="H68" s="2"/>
@@ -28977,7 +29096,7 @@
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
-      <c r="D69" s="32"/>
+      <c r="D69" s="31"/>
       <c r="E69" s="4"/>
       <c r="G69" s="1"/>
       <c r="H69" s="2"/>
@@ -28998,7 +29117,7 @@
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="32"/>
+      <c r="D70" s="31"/>
       <c r="E70" s="27"/>
       <c r="G70" s="1"/>
       <c r="H70" s="2"/>
@@ -29915,7 +30034,7 @@
       <c r="A4" s="28"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="34"/>
+      <c r="A5" s="33"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="15"/>
@@ -30002,7 +30121,7 @@
       <c r="B22" s="2" t="s">
         <v>1058</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="31" t="s">
         <v>1044</v>
       </c>
       <c r="D22" s="2" t="s">
@@ -30019,7 +30138,7 @@
       <c r="C23" s="2" t="s">
         <v>1048</v>
       </c>
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="31" t="s">
         <v>1047</v>
       </c>
     </row>
@@ -30033,7 +30152,7 @@
       <c r="C24" s="25" t="s">
         <v>1051</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="31" t="s">
         <v>1050</v>
       </c>
     </row>
@@ -30047,28 +30166,28 @@
       <c r="C25" s="2" t="s">
         <v>1054</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="31" t="s">
         <v>1053</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="C26" s="25"/>
-      <c r="D26" s="32"/>
+      <c r="D26" s="31"/>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="D28" s="32"/>
+      <c r="D28" s="31"/>
       <c r="E28" s="24"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="C29" s="25"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -30078,7 +30197,7 @@
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="C31" s="32"/>
+      <c r="C31" s="31"/>
       <c r="D31" s="2"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.3">
@@ -30090,92 +30209,92 @@
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="C33" s="25"/>
-      <c r="D33" s="32"/>
+      <c r="D33" s="31"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="C34" s="25"/>
-      <c r="D34" s="32"/>
+      <c r="D34" s="31"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="C35" s="25"/>
-      <c r="D35" s="32"/>
+      <c r="D35" s="31"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="C36" s="25"/>
-      <c r="D36" s="32"/>
+      <c r="D36" s="31"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="C37" s="25"/>
-      <c r="D37" s="32"/>
+      <c r="D37" s="31"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="C38" s="25"/>
-      <c r="D38" s="32"/>
+      <c r="D38" s="31"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
-      <c r="D39" s="32"/>
+      <c r="D39" s="31"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="C40" s="25"/>
-      <c r="D40" s="32"/>
+      <c r="D40" s="31"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="D41" s="32"/>
+      <c r="D41" s="31"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="C42" s="25"/>
-      <c r="D42" s="32"/>
+      <c r="D42" s="31"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="C43" s="25"/>
-      <c r="D43" s="32"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
-      <c r="D44" s="32"/>
+      <c r="D44" s="31"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="C45" s="25"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
-      <c r="D46" s="32"/>
+      <c r="D46" s="31"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D47" s="32"/>
+      <c r="D47" s="31"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D48" s="32"/>
+      <c r="D48" s="31"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="C49" s="25"/>
-      <c r="D49" s="32"/>
+      <c r="D49" s="31"/>
       <c r="E49" s="1"/>
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="C50" s="25"/>
-      <c r="D50" s="32"/>
+      <c r="D50" s="31"/>
       <c r="E50" s="1"/>
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="C51" s="25"/>
-      <c r="D51" s="32"/>
+      <c r="D51" s="31"/>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="C52" s="1"/>
@@ -30195,7 +30314,7 @@
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="25"/>
-      <c r="D53" s="32"/>
+      <c r="D53" s="31"/>
       <c r="E53" s="4"/>
       <c r="G53" s="1"/>
       <c r="H53" s="2"/>
@@ -30217,7 +30336,7 @@
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="25"/>
-      <c r="D55" s="32"/>
+      <c r="D55" s="31"/>
       <c r="E55" s="4"/>
       <c r="G55" s="1"/>
       <c r="H55" s="2"/>
@@ -30238,7 +30357,7 @@
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="25"/>
-      <c r="D56" s="32"/>
+      <c r="D56" s="31"/>
       <c r="E56" s="4"/>
       <c r="G56" s="1"/>
       <c r="H56" s="2"/>
@@ -30259,7 +30378,7 @@
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="25"/>
-      <c r="D57" s="32"/>
+      <c r="D57" s="31"/>
       <c r="E57" s="4"/>
       <c r="G57" s="1"/>
       <c r="H57" s="2"/>
@@ -30280,7 +30399,7 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="25"/>
-      <c r="D58" s="32"/>
+      <c r="D58" s="31"/>
       <c r="E58" s="4"/>
       <c r="G58" s="1"/>
       <c r="H58" s="2"/>
@@ -30301,7 +30420,7 @@
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="25"/>
-      <c r="D59" s="32"/>
+      <c r="D59" s="31"/>
       <c r="E59" s="4"/>
       <c r="G59" s="1"/>
       <c r="H59" s="2"/>
@@ -30322,7 +30441,7 @@
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="25"/>
-      <c r="D60" s="32"/>
+      <c r="D60" s="31"/>
       <c r="E60" s="4"/>
       <c r="G60" s="1"/>
       <c r="H60" s="2"/>
@@ -30343,7 +30462,7 @@
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="25"/>
-      <c r="D61" s="32"/>
+      <c r="D61" s="31"/>
       <c r="E61" s="4"/>
       <c r="G61" s="1"/>
       <c r="H61" s="2"/>
@@ -30364,7 +30483,7 @@
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="25"/>
-      <c r="D62" s="32"/>
+      <c r="D62" s="31"/>
       <c r="E62" s="4"/>
       <c r="G62" s="1"/>
       <c r="H62" s="2"/>
@@ -30385,7 +30504,7 @@
       <c r="A63" s="2"/>
       <c r="B63" s="27"/>
       <c r="C63" s="25"/>
-      <c r="D63" s="32"/>
+      <c r="D63" s="31"/>
       <c r="E63" s="4"/>
       <c r="G63" s="1"/>
       <c r="H63" s="2"/>
@@ -30406,7 +30525,7 @@
       <c r="A64" s="2"/>
       <c r="B64" s="27"/>
       <c r="C64" s="25"/>
-      <c r="D64" s="32"/>
+      <c r="D64" s="31"/>
       <c r="E64" s="4"/>
       <c r="G64" s="1"/>
       <c r="H64" s="2"/>
@@ -30427,7 +30546,7 @@
       <c r="A65" s="2"/>
       <c r="B65" s="27"/>
       <c r="C65" s="25"/>
-      <c r="D65" s="32"/>
+      <c r="D65" s="31"/>
       <c r="E65" s="4"/>
       <c r="G65" s="1"/>
       <c r="H65" s="2"/>
@@ -30448,7 +30567,7 @@
       <c r="A66" s="2"/>
       <c r="B66" s="27"/>
       <c r="C66" s="26"/>
-      <c r="D66" s="32"/>
+      <c r="D66" s="31"/>
       <c r="E66" s="4"/>
       <c r="G66" s="1"/>
       <c r="H66" s="2"/>
@@ -30469,7 +30588,7 @@
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
-      <c r="D67" s="32"/>
+      <c r="D67" s="31"/>
       <c r="E67" s="4"/>
       <c r="G67" s="1"/>
       <c r="H67" s="2"/>
@@ -30490,7 +30609,7 @@
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="25"/>
-      <c r="D68" s="32"/>
+      <c r="D68" s="31"/>
       <c r="E68" s="4"/>
       <c r="G68" s="1"/>
       <c r="H68" s="2"/>
@@ -30511,7 +30630,7 @@
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
-      <c r="D69" s="32"/>
+      <c r="D69" s="31"/>
       <c r="E69" s="4"/>
       <c r="G69" s="1"/>
       <c r="H69" s="2"/>
@@ -30532,7 +30651,7 @@
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="25"/>
-      <c r="D70" s="32"/>
+      <c r="D70" s="31"/>
       <c r="E70" s="27"/>
       <c r="G70" s="1"/>
       <c r="H70" s="2"/>

</xml_diff>